<commit_message>
updated input data file path
</commit_message>
<xml_diff>
--- a/RE-RPA Challenge/Data/Config.xlsx
+++ b/RE-RPA Challenge/Data/Config.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="18000" windowHeight="9480" activeTab="1"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="18000" windowHeight="9480"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -169,9 +169,6 @@
     <t>InputFilePath</t>
   </si>
   <si>
-    <t>H:\Projects\UiPath\RE-RPA Challenge\Data\Input\challenge.xlsx</t>
-  </si>
-  <si>
     <t>OrchestratorQueueName</t>
   </si>
   <si>
@@ -179,6 +176,9 @@
   </si>
   <si>
     <t>InputSheetName</t>
+  </si>
+  <si>
+    <t>Data\Input\challenge.xlsx</t>
   </si>
 </sst>
 </file>
@@ -604,7 +604,7 @@
     </row>
     <row r="2" spans="1:26">
       <c r="A2" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>46</v>
@@ -651,15 +651,15 @@
         <v>47</v>
       </c>
       <c r="B7" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:26">
       <c r="A8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>